<commit_message>
Update for version 7.0
</commit_message>
<xml_diff>
--- a/characters.xlsx
+++ b/characters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\genshinpuzzle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3218D185-28D7-4DFF-A981-9004F59320F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EF43DB-C3A0-417F-833B-CCD862F2C5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2BC2DB2F-00CC-4274-8DBF-E2A0BD6D3186}"/>
   </bookViews>
@@ -268,7 +268,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="209">
   <si>
     <t>Aino</t>
   </si>
@@ -857,6 +857,45 @@
   <si>
     <t>February 25, 2026</t>
   </si>
+  <si>
+    <t>Linnea</t>
+  </si>
+  <si>
+    <t>April 08, 2026</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>May 20, 2026</t>
+  </si>
+  <si>
+    <t>Prune</t>
+  </si>
+  <si>
+    <t>Lohen</t>
+  </si>
+  <si>
+    <t>June 09, 2026</t>
+  </si>
+  <si>
+    <t>Sandrone</t>
+  </si>
+  <si>
+    <t>July 01, 2026</t>
+  </si>
+  <si>
+    <t>Alyosha</t>
+  </si>
+  <si>
+    <t>August 12, 2026</t>
+  </si>
+  <si>
+    <t>Odette</t>
+  </si>
+  <si>
+    <t>Traveler (Cryo)</t>
+  </si>
 </sst>
 </file>
 
@@ -53063,7 +53102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82BBB357-DBD0-43D1-9851-C679B1E8E460}">
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:K127"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -54538,6 +54577,94 @@
         <v>195</v>
       </c>
     </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>196</v>
+      </c>
+      <c r="B120" t="s">
+        <v>3</v>
+      </c>
+      <c r="C120" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>198</v>
+      </c>
+      <c r="B121" t="s">
+        <v>9</v>
+      </c>
+      <c r="C121" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>200</v>
+      </c>
+      <c r="B122" t="s">
+        <v>20</v>
+      </c>
+      <c r="C122" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>201</v>
+      </c>
+      <c r="B123" t="s">
+        <v>7</v>
+      </c>
+      <c r="C123" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>203</v>
+      </c>
+      <c r="B124" t="s">
+        <v>7</v>
+      </c>
+      <c r="C124" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>205</v>
+      </c>
+      <c r="B125" t="s">
+        <v>15</v>
+      </c>
+      <c r="C125" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>207</v>
+      </c>
+      <c r="B126" t="s">
+        <v>7</v>
+      </c>
+      <c r="C126" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>208</v>
+      </c>
+      <c r="B127" t="s">
+        <v>7</v>
+      </c>
+      <c r="C127" t="s">
+        <v>206</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="K92:K95"/>

</xml_diff>

<commit_message>
Adding auto detect for daily/endless
</commit_message>
<xml_diff>
--- a/characters.xlsx
+++ b/characters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\genshinpuzzle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EF43DB-C3A0-417F-833B-CCD862F2C5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC83CA6-9B37-4A8E-B046-7A2170F6E69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2BC2DB2F-00CC-4274-8DBF-E2A0BD6D3186}"/>
   </bookViews>
@@ -35,240 +35,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="22">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="2"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="6"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="7"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="8"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="9"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="10"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="11"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="12"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="13"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="14"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="15"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="16"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="17"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="18"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="19"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="20"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="21"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="22">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-    <bk>
-      <rc t="1" v="2"/>
-    </bk>
-    <bk>
-      <rc t="1" v="3"/>
-    </bk>
-    <bk>
-      <rc t="1" v="4"/>
-    </bk>
-    <bk>
-      <rc t="1" v="5"/>
-    </bk>
-    <bk>
-      <rc t="1" v="6"/>
-    </bk>
-    <bk>
-      <rc t="1" v="7"/>
-    </bk>
-    <bk>
-      <rc t="1" v="8"/>
-    </bk>
-    <bk>
-      <rc t="1" v="9"/>
-    </bk>
-    <bk>
-      <rc t="1" v="10"/>
-    </bk>
-    <bk>
-      <rc t="1" v="11"/>
-    </bk>
-    <bk>
-      <rc t="1" v="12"/>
-    </bk>
-    <bk>
-      <rc t="1" v="13"/>
-    </bk>
-    <bk>
-      <rc t="1" v="14"/>
-    </bk>
-    <bk>
-      <rc t="1" v="15"/>
-    </bk>
-    <bk>
-      <rc t="1" v="16"/>
-    </bk>
-    <bk>
-      <rc t="1" v="17"/>
-    </bk>
-    <bk>
-      <rc t="1" v="18"/>
-    </bk>
-    <bk>
-      <rc t="1" v="19"/>
-    </bk>
-    <bk>
-      <rc t="1" v="20"/>
-    </bk>
-    <bk>
-      <rc t="1" v="21"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="212">
   <si>
     <t>Aino</t>
   </si>
@@ -896,6 +664,15 @@
   <si>
     <t>Traveler (Cryo)</t>
   </si>
+  <si>
+    <t>rarity</t>
+  </si>
+  <si>
+    <t>standard</t>
+  </si>
+  <si>
+    <t>temper</t>
+  </si>
 </sst>
 </file>
 
@@ -27236,13 +27013,13 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>209550</xdr:rowOff>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>600075</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -27259,7 +27036,7 @@
       </xdr:nvSpPr>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="8629650" y="1733550"/>
+          <a:off x="5124450" y="942975"/>
           <a:ext cx="600075" cy="152400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -52612,177 +52389,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="22">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Kaveh Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Keqing Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Kinich Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Kirara Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Klee Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Kujou Sara Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Kuki Shinobu Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Lan Yan Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Lauma Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Layla Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Lisa Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Lynette Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Qiqi Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Rosaria Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Sangonomiya Kokomi Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Shenhe Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Shikanoin Heizou Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Sigewinne Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Skirk Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Sucrose Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Tartaglia Icon</v>
-  </rv>
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-    <v>Thoma Icon</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-    <k n="Text" t="s"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -53118,6 +52724,15 @@
       <c r="C1" t="s">
         <v>187</v>
       </c>
+      <c r="E1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F1" t="s">
+        <v>210</v>
+      </c>
+      <c r="G1" t="s">
+        <v>211</v>
+      </c>
       <c r="K1" s="1"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -53130,6 +52745,15 @@
       <c r="C2" t="s">
         <v>121</v>
       </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -53142,6 +52766,15 @@
       <c r="C3" t="s">
         <v>122</v>
       </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -53154,6 +52787,15 @@
       <c r="C4" t="s">
         <v>123</v>
       </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
       <c r="K4" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -53166,6 +52808,15 @@
       <c r="C5" t="s">
         <v>124</v>
       </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
       <c r="K5" s="1"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -53178,6 +52829,15 @@
       <c r="C6" t="s">
         <v>125</v>
       </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
       <c r="K6" s="1"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -53190,6 +52850,15 @@
       <c r="C7" t="s">
         <v>126</v>
       </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
       <c r="K7" s="1"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -53202,6 +52871,15 @@
       <c r="C8" t="s">
         <v>127</v>
       </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
       <c r="K8" s="1"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -53214,6 +52892,15 @@
       <c r="C9" t="s">
         <v>128</v>
       </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
       <c r="K9" s="1"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -53226,6 +52913,15 @@
       <c r="C10" t="s">
         <v>125</v>
       </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
       <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -53238,6 +52934,15 @@
       <c r="C11" t="s">
         <v>125</v>
       </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
       <c r="K11" s="1"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -53250,6 +52955,15 @@
       <c r="C12" t="s">
         <v>125</v>
       </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
       <c r="K12" s="1"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -53262,6 +52976,15 @@
       <c r="C13" t="s">
         <v>129</v>
       </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
       <c r="K13" s="1"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -53274,6 +52997,15 @@
       <c r="C14" t="s">
         <v>130</v>
       </c>
+      <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
       <c r="K14" s="1"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -53286,6 +53018,15 @@
       <c r="C15" t="s">
         <v>131</v>
       </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
       <c r="K15" s="1"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -53298,6 +53039,15 @@
       <c r="C16" t="s">
         <v>132</v>
       </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
       <c r="K16" s="1"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -53310,6 +53060,15 @@
       <c r="C17" t="s">
         <v>133</v>
       </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+      <c r="F17" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
       <c r="K17" s="1"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -53322,6 +53081,15 @@
       <c r="C18" t="s">
         <v>125</v>
       </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
       <c r="K18" s="1"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -53334,6 +53102,15 @@
       <c r="C19" t="s">
         <v>134</v>
       </c>
+      <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19" t="b">
+        <v>0</v>
+      </c>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
       <c r="K19" s="1"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -53346,6 +53123,15 @@
       <c r="C20" t="s">
         <v>135</v>
       </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
       <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -53358,6 +53144,15 @@
       <c r="C21" t="s">
         <v>136</v>
       </c>
+      <c r="E21">
+        <v>4</v>
+      </c>
+      <c r="F21" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
       <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -53370,6 +53165,15 @@
       <c r="C22" t="s">
         <v>137</v>
       </c>
+      <c r="E22">
+        <v>5</v>
+      </c>
+      <c r="F22" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
       <c r="K22" s="1"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -53382,6 +53186,15 @@
       <c r="C23" t="s">
         <v>129</v>
       </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+      <c r="F23" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
       <c r="K23" s="1"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -53394,6 +53207,15 @@
       <c r="C24" t="s">
         <v>138</v>
       </c>
+      <c r="E24">
+        <v>4</v>
+      </c>
+      <c r="F24" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
       <c r="K24" s="1"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -53406,6 +53228,15 @@
       <c r="C25" t="s">
         <v>139</v>
       </c>
+      <c r="E25">
+        <v>5</v>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
       <c r="K25" s="1"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -53418,6 +53249,15 @@
       <c r="C26" t="s">
         <v>125</v>
       </c>
+      <c r="E26">
+        <v>5</v>
+      </c>
+      <c r="F26" t="b">
+        <v>1</v>
+      </c>
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
       <c r="K26" s="1"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -53430,6 +53270,15 @@
       <c r="C27" t="s">
         <v>140</v>
       </c>
+      <c r="E27">
+        <v>4</v>
+      </c>
+      <c r="F27" t="b">
+        <v>0</v>
+      </c>
+      <c r="G27" t="b">
+        <v>0</v>
+      </c>
       <c r="K27" s="1"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -53442,6 +53291,15 @@
       <c r="C28" t="s">
         <v>141</v>
       </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" t="b">
+        <v>0</v>
+      </c>
       <c r="K28" s="1"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -53454,6 +53312,15 @@
       <c r="C29" t="s">
         <v>142</v>
       </c>
+      <c r="E29">
+        <v>5</v>
+      </c>
+      <c r="F29" t="b">
+        <v>0</v>
+      </c>
+      <c r="G29" t="b">
+        <v>0</v>
+      </c>
       <c r="K29" s="1"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -53466,6 +53333,15 @@
       <c r="C30" t="s">
         <v>143</v>
       </c>
+      <c r="E30">
+        <v>5</v>
+      </c>
+      <c r="F30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
       <c r="K30" s="1"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -53478,6 +53354,15 @@
       <c r="C31" t="s">
         <v>144</v>
       </c>
+      <c r="E31">
+        <v>5</v>
+      </c>
+      <c r="F31" t="b">
+        <v>0</v>
+      </c>
+      <c r="G31" t="b">
+        <v>0</v>
+      </c>
       <c r="K31" s="1"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -53490,6 +53375,15 @@
       <c r="C32" t="s">
         <v>145</v>
       </c>
+      <c r="E32">
+        <v>5</v>
+      </c>
+      <c r="F32" t="b">
+        <v>0</v>
+      </c>
+      <c r="G32" t="b">
+        <v>1</v>
+      </c>
       <c r="K32" s="1"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -53502,6 +53396,15 @@
       <c r="C33" t="s">
         <v>146</v>
       </c>
+      <c r="E33">
+        <v>4</v>
+      </c>
+      <c r="F33" t="b">
+        <v>0</v>
+      </c>
+      <c r="G33" t="b">
+        <v>0</v>
+      </c>
       <c r="K33" s="1"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -53514,6 +53417,15 @@
       <c r="C34" t="s">
         <v>125</v>
       </c>
+      <c r="E34">
+        <v>4</v>
+      </c>
+      <c r="F34" t="b">
+        <v>0</v>
+      </c>
+      <c r="G34" t="b">
+        <v>0</v>
+      </c>
       <c r="K34" s="1"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -53526,6 +53438,15 @@
       <c r="C35" t="s">
         <v>147</v>
       </c>
+      <c r="E35">
+        <v>5</v>
+      </c>
+      <c r="F35" t="b">
+        <v>0</v>
+      </c>
+      <c r="G35" t="b">
+        <v>0</v>
+      </c>
       <c r="K35" s="1"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -53538,6 +53459,15 @@
       <c r="C36" t="s">
         <v>148</v>
       </c>
+      <c r="E36">
+        <v>4</v>
+      </c>
+      <c r="F36" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36" t="b">
+        <v>0</v>
+      </c>
       <c r="K36" s="1"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -53550,6 +53480,15 @@
       <c r="C37" t="s">
         <v>130</v>
       </c>
+      <c r="E37">
+        <v>5</v>
+      </c>
+      <c r="F37" t="b">
+        <v>0</v>
+      </c>
+      <c r="G37" t="b">
+        <v>0</v>
+      </c>
       <c r="K37" s="1"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -53562,6 +53501,15 @@
       <c r="C38" t="s">
         <v>149</v>
       </c>
+      <c r="E38">
+        <v>4</v>
+      </c>
+      <c r="F38" t="b">
+        <v>0</v>
+      </c>
+      <c r="G38" t="b">
+        <v>0</v>
+      </c>
       <c r="K38" s="1"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -53574,6 +53522,15 @@
       <c r="C39" t="s">
         <v>150</v>
       </c>
+      <c r="E39">
+        <v>5</v>
+      </c>
+      <c r="F39" t="b">
+        <v>0</v>
+      </c>
+      <c r="G39" t="b">
+        <v>1</v>
+      </c>
       <c r="K39" s="1"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -53586,6 +53543,15 @@
       <c r="C40" t="s">
         <v>126</v>
       </c>
+      <c r="E40">
+        <v>4</v>
+      </c>
+      <c r="F40" t="b">
+        <v>0</v>
+      </c>
+      <c r="G40" t="b">
+        <v>0</v>
+      </c>
       <c r="K40" s="1"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -53598,6 +53564,15 @@
       <c r="C41" t="s">
         <v>151</v>
       </c>
+      <c r="E41">
+        <v>5</v>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+      <c r="G41" t="b">
+        <v>1</v>
+      </c>
       <c r="K41" s="1"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -53610,6 +53585,15 @@
       <c r="C42" t="s">
         <v>152</v>
       </c>
+      <c r="E42">
+        <v>4</v>
+      </c>
+      <c r="F42" t="b">
+        <v>0</v>
+      </c>
+      <c r="G42" t="b">
+        <v>0</v>
+      </c>
       <c r="K42" s="1"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -53622,6 +53606,15 @@
       <c r="C43" t="s">
         <v>144</v>
       </c>
+      <c r="E43">
+        <v>4</v>
+      </c>
+      <c r="F43" t="b">
+        <v>0</v>
+      </c>
+      <c r="G43" t="b">
+        <v>0</v>
+      </c>
       <c r="K43" s="1"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -53634,6 +53627,15 @@
       <c r="C44" t="s">
         <v>153</v>
       </c>
+      <c r="E44">
+        <v>4</v>
+      </c>
+      <c r="F44" t="b">
+        <v>0</v>
+      </c>
+      <c r="G44" t="b">
+        <v>0</v>
+      </c>
       <c r="K44" s="1"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -53646,6 +53648,15 @@
       <c r="C45" t="s">
         <v>154</v>
       </c>
+      <c r="E45">
+        <v>5</v>
+      </c>
+      <c r="F45" t="b">
+        <v>0</v>
+      </c>
+      <c r="G45" t="b">
+        <v>0</v>
+      </c>
       <c r="K45" s="1"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -53658,6 +53669,15 @@
       <c r="C46" t="s">
         <v>142</v>
       </c>
+      <c r="E46">
+        <v>4</v>
+      </c>
+      <c r="F46" t="b">
+        <v>0</v>
+      </c>
+      <c r="G46" t="b">
+        <v>0</v>
+      </c>
       <c r="K46" s="1"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -53670,6 +53690,15 @@
       <c r="C47" t="s">
         <v>125</v>
       </c>
+      <c r="E47">
+        <v>5</v>
+      </c>
+      <c r="F47" t="b">
+        <v>1</v>
+      </c>
+      <c r="G47" t="b">
+        <v>0</v>
+      </c>
       <c r="K47" s="1"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -53682,6 +53711,15 @@
       <c r="C48" t="s">
         <v>155</v>
       </c>
+      <c r="E48">
+        <v>4</v>
+      </c>
+      <c r="F48" t="b">
+        <v>0</v>
+      </c>
+      <c r="G48" t="b">
+        <v>0</v>
+      </c>
       <c r="K48" s="1"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -53694,6 +53732,15 @@
       <c r="C49" t="s">
         <v>156</v>
       </c>
+      <c r="E49">
+        <v>5</v>
+      </c>
+      <c r="F49" t="b">
+        <v>0</v>
+      </c>
+      <c r="G49" t="b">
+        <v>0</v>
+      </c>
       <c r="K49" s="1"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -53706,6 +53753,15 @@
       <c r="C50" t="s">
         <v>125</v>
       </c>
+      <c r="E50">
+        <v>4</v>
+      </c>
+      <c r="F50" t="b">
+        <v>0</v>
+      </c>
+      <c r="G50" t="b">
+        <v>0</v>
+      </c>
       <c r="K50" s="1"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -53718,6 +53774,15 @@
       <c r="C51" t="s">
         <v>157</v>
       </c>
+      <c r="E51">
+        <v>5</v>
+      </c>
+      <c r="F51" t="b">
+        <v>0</v>
+      </c>
+      <c r="G51" t="b">
+        <v>1</v>
+      </c>
       <c r="K51" s="1"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -53730,9 +53795,16 @@
       <c r="C52" t="s">
         <v>158</v>
       </c>
-      <c r="K52" s="1" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E52">
+        <v>5</v>
+      </c>
+      <c r="F52" t="b">
+        <v>0</v>
+      </c>
+      <c r="G52" t="b">
+        <v>1</v>
+      </c>
+      <c r="K52" s="1"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -53744,9 +53816,16 @@
       <c r="C53" t="s">
         <v>128</v>
       </c>
-      <c r="K53" s="1" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E53">
+        <v>4</v>
+      </c>
+      <c r="F53" t="b">
+        <v>0</v>
+      </c>
+      <c r="G53" t="b">
+        <v>0</v>
+      </c>
+      <c r="K53" s="1"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -53758,9 +53837,16 @@
       <c r="C54" t="s">
         <v>125</v>
       </c>
-      <c r="K54" s="1" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E54">
+        <v>5</v>
+      </c>
+      <c r="F54" t="b">
+        <v>1</v>
+      </c>
+      <c r="G54" t="b">
+        <v>0</v>
+      </c>
+      <c r="K54" s="1"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
@@ -53772,9 +53858,16 @@
       <c r="C55" t="s">
         <v>159</v>
       </c>
-      <c r="K55" s="1" t="e" vm="4">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E55">
+        <v>5</v>
+      </c>
+      <c r="F55" t="b">
+        <v>0</v>
+      </c>
+      <c r="G55" t="b">
+        <v>0</v>
+      </c>
+      <c r="K55" s="1"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
@@ -53786,9 +53879,16 @@
       <c r="C56" t="s">
         <v>160</v>
       </c>
-      <c r="K56" s="1" t="e" vm="5">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E56">
+        <v>4</v>
+      </c>
+      <c r="F56" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" t="b">
+        <v>0</v>
+      </c>
+      <c r="K56" s="1"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
@@ -53800,9 +53900,16 @@
       <c r="C57" t="s">
         <v>161</v>
       </c>
-      <c r="K57" s="1" t="e" vm="6">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E57">
+        <v>5</v>
+      </c>
+      <c r="F57" t="b">
+        <v>0</v>
+      </c>
+      <c r="G57" t="b">
+        <v>1</v>
+      </c>
+      <c r="K57" s="1"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -53814,9 +53921,16 @@
       <c r="C58" t="s">
         <v>124</v>
       </c>
-      <c r="K58" s="1" t="e" vm="7">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E58">
+        <v>4</v>
+      </c>
+      <c r="F58" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" t="b">
+        <v>0</v>
+      </c>
+      <c r="K58" s="1"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
@@ -53828,9 +53942,16 @@
       <c r="C59" t="s">
         <v>162</v>
       </c>
-      <c r="K59" s="1" t="e" vm="8">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E59">
+        <v>4</v>
+      </c>
+      <c r="F59" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" t="b">
+        <v>0</v>
+      </c>
+      <c r="K59" s="1"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
@@ -53842,9 +53963,16 @@
       <c r="C60" t="s">
         <v>163</v>
       </c>
-      <c r="K60" s="1" t="e" vm="9">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E60">
+        <v>4</v>
+      </c>
+      <c r="F60" t="b">
+        <v>0</v>
+      </c>
+      <c r="G60" t="b">
+        <v>0</v>
+      </c>
+      <c r="K60" s="1"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
@@ -53856,9 +53984,16 @@
       <c r="C61" t="s">
         <v>121</v>
       </c>
-      <c r="K61" s="1" t="e" vm="10">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E61">
+        <v>5</v>
+      </c>
+      <c r="F61" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" t="b">
+        <v>0</v>
+      </c>
+      <c r="K61" s="1"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
@@ -53870,9 +54005,16 @@
       <c r="C62" t="s">
         <v>164</v>
       </c>
-      <c r="K62" s="1" t="e" vm="11">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E62">
+        <v>4</v>
+      </c>
+      <c r="F62" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" t="b">
+        <v>0</v>
+      </c>
+      <c r="K62" s="1"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
@@ -53884,9 +54026,16 @@
       <c r="C63" t="s">
         <v>125</v>
       </c>
-      <c r="K63" s="1" t="e" vm="12">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E63">
+        <v>4</v>
+      </c>
+      <c r="F63" t="b">
+        <v>0</v>
+      </c>
+      <c r="G63" t="b">
+        <v>0</v>
+      </c>
+      <c r="K63" s="1"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
@@ -53897,6 +54046,15 @@
       </c>
       <c r="C64" t="s">
         <v>165</v>
+      </c>
+      <c r="E64">
+        <v>4</v>
+      </c>
+      <c r="F64" t="b">
+        <v>0</v>
+      </c>
+      <c r="G64" t="b">
+        <v>0</v>
       </c>
       <c r="K64" s="1"/>
     </row>
@@ -53910,6 +54068,15 @@
       <c r="C65" t="s">
         <v>165</v>
       </c>
+      <c r="E65">
+        <v>5</v>
+      </c>
+      <c r="F65" t="b">
+        <v>0</v>
+      </c>
+      <c r="G65" t="b">
+        <v>1</v>
+      </c>
       <c r="K65" s="1"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -53922,6 +54089,15 @@
       <c r="C66" t="s">
         <v>134</v>
       </c>
+      <c r="E66">
+        <v>5</v>
+      </c>
+      <c r="F66" t="b">
+        <v>0</v>
+      </c>
+      <c r="G66" t="b">
+        <v>0</v>
+      </c>
       <c r="K66" s="1"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -53934,6 +54110,15 @@
       <c r="C67" t="s">
         <v>166</v>
       </c>
+      <c r="E67">
+        <v>4</v>
+      </c>
+      <c r="F67" t="b">
+        <v>0</v>
+      </c>
+      <c r="G67" t="b">
+        <v>0</v>
+      </c>
       <c r="K67" s="1"/>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -53946,6 +54131,15 @@
       <c r="C68" t="s">
         <v>125</v>
       </c>
+      <c r="E68">
+        <v>5</v>
+      </c>
+      <c r="F68" t="b">
+        <v>1</v>
+      </c>
+      <c r="G68" t="b">
+        <v>0</v>
+      </c>
       <c r="K68" s="1"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -53958,6 +54152,15 @@
       <c r="C69" t="s">
         <v>155</v>
       </c>
+      <c r="E69">
+        <v>5</v>
+      </c>
+      <c r="F69" t="b">
+        <v>0</v>
+      </c>
+      <c r="G69" t="b">
+        <v>0</v>
+      </c>
       <c r="K69" s="1"/>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -53970,6 +54173,15 @@
       <c r="C70" t="s">
         <v>167</v>
       </c>
+      <c r="E70">
+        <v>5</v>
+      </c>
+      <c r="F70" t="b">
+        <v>0</v>
+      </c>
+      <c r="G70" t="b">
+        <v>0</v>
+      </c>
       <c r="K70" s="1"/>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -53982,6 +54194,15 @@
       <c r="C71" t="s">
         <v>168</v>
       </c>
+      <c r="E71">
+        <v>5</v>
+      </c>
+      <c r="F71" t="b">
+        <v>0</v>
+      </c>
+      <c r="G71" t="b">
+        <v>1</v>
+      </c>
       <c r="K71" s="1"/>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -53994,6 +54215,15 @@
       <c r="C72" t="s">
         <v>169</v>
       </c>
+      <c r="E72">
+        <v>5</v>
+      </c>
+      <c r="F72" t="b">
+        <v>0</v>
+      </c>
+      <c r="G72" t="b">
+        <v>0</v>
+      </c>
       <c r="K72" s="1"/>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -54006,6 +54236,15 @@
       <c r="C73" t="s">
         <v>170</v>
       </c>
+      <c r="E73">
+        <v>5</v>
+      </c>
+      <c r="F73" t="b">
+        <v>0</v>
+      </c>
+      <c r="G73" t="b">
+        <v>0</v>
+      </c>
       <c r="K73" s="1"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -54018,6 +54257,15 @@
       <c r="C74" t="s">
         <v>171</v>
       </c>
+      <c r="E74">
+        <v>5</v>
+      </c>
+      <c r="F74" t="b">
+        <v>0</v>
+      </c>
+      <c r="G74" t="b">
+        <v>1</v>
+      </c>
       <c r="K74" s="1"/>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -54030,6 +54278,15 @@
       <c r="C75" t="s">
         <v>125</v>
       </c>
+      <c r="E75">
+        <v>4</v>
+      </c>
+      <c r="F75" t="b">
+        <v>0</v>
+      </c>
+      <c r="G75" t="b">
+        <v>0</v>
+      </c>
       <c r="K75" s="1"/>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -54042,6 +54299,15 @@
       <c r="C76" t="s">
         <v>125</v>
       </c>
+      <c r="E76">
+        <v>4</v>
+      </c>
+      <c r="F76" t="b">
+        <v>0</v>
+      </c>
+      <c r="G76" t="b">
+        <v>0</v>
+      </c>
       <c r="K76" s="1"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
@@ -54054,9 +54320,16 @@
       <c r="C77" t="s">
         <v>131</v>
       </c>
-      <c r="K77" s="1" t="e" vm="13">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E77">
+        <v>4</v>
+      </c>
+      <c r="F77" t="b">
+        <v>0</v>
+      </c>
+      <c r="G77" t="b">
+        <v>0</v>
+      </c>
+      <c r="K77" s="1"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
@@ -54067,6 +54340,15 @@
       </c>
       <c r="C78" t="s">
         <v>125</v>
+      </c>
+      <c r="E78">
+        <v>5</v>
+      </c>
+      <c r="F78" t="b">
+        <v>1</v>
+      </c>
+      <c r="G78" t="b">
+        <v>0</v>
       </c>
       <c r="K78" s="1"/>
     </row>
@@ -54080,6 +54362,15 @@
       <c r="C79" t="s">
         <v>124</v>
       </c>
+      <c r="E79">
+        <v>5</v>
+      </c>
+      <c r="F79" t="b">
+        <v>0</v>
+      </c>
+      <c r="G79" t="b">
+        <v>0</v>
+      </c>
       <c r="K79" s="1"/>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -54092,9 +54383,16 @@
       <c r="C80" t="s">
         <v>125</v>
       </c>
-      <c r="K80" s="1" t="e" vm="14">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E80">
+        <v>4</v>
+      </c>
+      <c r="F80" t="b">
+        <v>0</v>
+      </c>
+      <c r="G80" t="b">
+        <v>0</v>
+      </c>
+      <c r="K80" s="1"/>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
@@ -54106,9 +54404,16 @@
       <c r="C81" t="s">
         <v>172</v>
       </c>
-      <c r="K81" s="1" t="e" vm="15">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E81">
+        <v>4</v>
+      </c>
+      <c r="F81" t="b">
+        <v>0</v>
+      </c>
+      <c r="G81" t="b">
+        <v>0</v>
+      </c>
+      <c r="K81" s="1"/>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
@@ -54119,6 +54424,15 @@
       </c>
       <c r="C82" t="s">
         <v>173</v>
+      </c>
+      <c r="E82">
+        <v>5</v>
+      </c>
+      <c r="F82" t="b">
+        <v>0</v>
+      </c>
+      <c r="G82" t="b">
+        <v>1</v>
       </c>
       <c r="K82" s="1"/>
     </row>
@@ -54132,6 +54446,15 @@
       <c r="C83" t="s">
         <v>174</v>
       </c>
+      <c r="E83">
+        <v>4</v>
+      </c>
+      <c r="F83" t="b">
+        <v>0</v>
+      </c>
+      <c r="G83" t="b">
+        <v>0</v>
+      </c>
       <c r="K83" s="1"/>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -54144,9 +54467,16 @@
       <c r="C84" t="s">
         <v>135</v>
       </c>
-      <c r="K84" s="1" t="e" vm="16">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E84">
+        <v>4</v>
+      </c>
+      <c r="F84" t="b">
+        <v>0</v>
+      </c>
+      <c r="G84" t="b">
+        <v>0</v>
+      </c>
+      <c r="K84" s="1"/>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
@@ -54158,9 +54488,16 @@
       <c r="C85" t="s">
         <v>175</v>
       </c>
-      <c r="K85" s="1" t="e" vm="17">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E85">
+        <v>5</v>
+      </c>
+      <c r="F85" t="b">
+        <v>0</v>
+      </c>
+      <c r="G85" t="b">
+        <v>1</v>
+      </c>
+      <c r="K85" s="1"/>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
@@ -54172,9 +54509,16 @@
       <c r="C86" t="s">
         <v>176</v>
       </c>
-      <c r="K86" s="1" t="e" vm="18">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E86">
+        <v>4</v>
+      </c>
+      <c r="F86" t="b">
+        <v>0</v>
+      </c>
+      <c r="G86" t="b">
+        <v>0</v>
+      </c>
+      <c r="K86" s="1"/>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
@@ -54186,9 +54530,16 @@
       <c r="C87" t="s">
         <v>177</v>
       </c>
-      <c r="K87" s="1" t="e" vm="19">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E87">
+        <v>5</v>
+      </c>
+      <c r="F87" t="b">
+        <v>0</v>
+      </c>
+      <c r="G87" t="b">
+        <v>1</v>
+      </c>
+      <c r="K87" s="1"/>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
@@ -54200,9 +54551,16 @@
       <c r="C88" t="s">
         <v>138</v>
       </c>
-      <c r="K88" s="1" t="e" vm="20">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E88">
+        <v>5</v>
+      </c>
+      <c r="F88" t="b">
+        <v>0</v>
+      </c>
+      <c r="G88" t="b">
+        <v>0</v>
+      </c>
+      <c r="K88" s="1"/>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
@@ -54214,9 +54572,16 @@
       <c r="C89" t="s">
         <v>125</v>
       </c>
-      <c r="K89" s="1" t="e" vm="21">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E89">
+        <v>4</v>
+      </c>
+      <c r="F89" t="b">
+        <v>0</v>
+      </c>
+      <c r="G89" t="b">
+        <v>0</v>
+      </c>
+      <c r="K89" s="1"/>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
@@ -54228,9 +54593,16 @@
       <c r="C90" t="s">
         <v>140</v>
       </c>
-      <c r="K90" s="1" t="e" vm="22">
-        <v>#VALUE!</v>
-      </c>
+      <c r="E90">
+        <v>5</v>
+      </c>
+      <c r="F90" t="b">
+        <v>0</v>
+      </c>
+      <c r="G90" t="b">
+        <v>1</v>
+      </c>
+      <c r="K90" s="1"/>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
@@ -54241,6 +54613,15 @@
       </c>
       <c r="C91" t="s">
         <v>178</v>
+      </c>
+      <c r="E91">
+        <v>4</v>
+      </c>
+      <c r="F91" t="b">
+        <v>0</v>
+      </c>
+      <c r="G91" t="b">
+        <v>0</v>
       </c>
       <c r="K91" s="1"/>
     </row>
@@ -54254,6 +54635,15 @@
       <c r="C92" t="s">
         <v>136</v>
       </c>
+      <c r="E92">
+        <v>5</v>
+      </c>
+      <c r="F92" t="b">
+        <v>1</v>
+      </c>
+      <c r="G92" t="b">
+        <v>0</v>
+      </c>
       <c r="K92" s="2"/>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
@@ -54266,6 +54656,15 @@
       <c r="C93" t="s">
         <v>125</v>
       </c>
+      <c r="E93">
+        <v>4</v>
+      </c>
+      <c r="F93" t="b">
+        <v>0</v>
+      </c>
+      <c r="G93" t="b">
+        <v>0</v>
+      </c>
       <c r="K93" s="2"/>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
@@ -54278,6 +54677,15 @@
       <c r="C94" t="s">
         <v>125</v>
       </c>
+      <c r="E94">
+        <v>4</v>
+      </c>
+      <c r="F94" t="b">
+        <v>0</v>
+      </c>
+      <c r="G94" t="b">
+        <v>0</v>
+      </c>
       <c r="K94" s="2"/>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.25">
@@ -54290,6 +54698,15 @@
       <c r="C95" t="s">
         <v>174</v>
       </c>
+      <c r="E95">
+        <v>4</v>
+      </c>
+      <c r="F95" t="b">
+        <v>0</v>
+      </c>
+      <c r="G95" t="b">
+        <v>0</v>
+      </c>
       <c r="K95" s="2"/>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
@@ -54302,6 +54719,15 @@
       <c r="C96" t="s">
         <v>136</v>
       </c>
+      <c r="E96">
+        <v>4</v>
+      </c>
+      <c r="F96" t="b">
+        <v>0</v>
+      </c>
+      <c r="G96" t="b">
+        <v>0</v>
+      </c>
       <c r="K96" s="1"/>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
@@ -54314,6 +54740,15 @@
       <c r="C97" t="s">
         <v>165</v>
       </c>
+      <c r="E97">
+        <v>4</v>
+      </c>
+      <c r="F97" t="b">
+        <v>0</v>
+      </c>
+      <c r="G97" t="b">
+        <v>0</v>
+      </c>
       <c r="K97" s="1"/>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
@@ -54326,6 +54761,15 @@
       <c r="C98" t="s">
         <v>134</v>
       </c>
+      <c r="E98">
+        <v>4</v>
+      </c>
+      <c r="F98" t="b">
+        <v>0</v>
+      </c>
+      <c r="G98" t="b">
+        <v>0</v>
+      </c>
       <c r="K98" s="1"/>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
@@ -54338,6 +54782,15 @@
       <c r="C99" t="s">
         <v>125</v>
       </c>
+      <c r="E99">
+        <v>4</v>
+      </c>
+      <c r="F99" t="b">
+        <v>0</v>
+      </c>
+      <c r="G99" t="b">
+        <v>0</v>
+      </c>
       <c r="K99" s="1"/>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -54350,6 +54803,15 @@
       <c r="C100" t="s">
         <v>152</v>
       </c>
+      <c r="E100">
+        <v>5</v>
+      </c>
+      <c r="F100" t="b">
+        <v>0</v>
+      </c>
+      <c r="G100" t="b">
+        <v>0</v>
+      </c>
       <c r="K100" s="1"/>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
@@ -54362,6 +54824,15 @@
       <c r="C101" t="s">
         <v>125</v>
       </c>
+      <c r="E101">
+        <v>5</v>
+      </c>
+      <c r="F101" t="b">
+        <v>0</v>
+      </c>
+      <c r="G101" t="b">
+        <v>0</v>
+      </c>
       <c r="K101" s="1"/>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -54374,6 +54845,15 @@
       <c r="C102" t="s">
         <v>146</v>
       </c>
+      <c r="E102">
+        <v>5</v>
+      </c>
+      <c r="F102" t="b">
+        <v>0</v>
+      </c>
+      <c r="G102" t="b">
+        <v>1</v>
+      </c>
       <c r="K102" s="1"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
@@ -54386,6 +54866,15 @@
       <c r="C103" t="s">
         <v>179</v>
       </c>
+      <c r="E103">
+        <v>5</v>
+      </c>
+      <c r="F103" t="b">
+        <v>0</v>
+      </c>
+      <c r="G103" t="b">
+        <v>1</v>
+      </c>
       <c r="K103" s="1"/>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
@@ -54398,6 +54887,15 @@
       <c r="C104" t="s">
         <v>125</v>
       </c>
+      <c r="E104">
+        <v>4</v>
+      </c>
+      <c r="F104" t="b">
+        <v>0</v>
+      </c>
+      <c r="G104" t="b">
+        <v>0</v>
+      </c>
       <c r="K104" s="1"/>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
@@ -54410,6 +54908,15 @@
       <c r="C105" t="s">
         <v>149</v>
       </c>
+      <c r="E105">
+        <v>5</v>
+      </c>
+      <c r="F105" t="b">
+        <v>0</v>
+      </c>
+      <c r="G105" t="b">
+        <v>1</v>
+      </c>
       <c r="K105" s="1"/>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
@@ -54422,6 +54929,15 @@
       <c r="C106" t="s">
         <v>180</v>
       </c>
+      <c r="E106">
+        <v>5</v>
+      </c>
+      <c r="F106" t="b">
+        <v>0</v>
+      </c>
+      <c r="G106" t="b">
+        <v>1</v>
+      </c>
       <c r="K106" s="1"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
@@ -54434,6 +54950,15 @@
       <c r="C107" t="s">
         <v>181</v>
       </c>
+      <c r="E107">
+        <v>5</v>
+      </c>
+      <c r="F107" t="b">
+        <v>0</v>
+      </c>
+      <c r="G107" t="b">
+        <v>0</v>
+      </c>
       <c r="K107" s="1"/>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
@@ -54446,6 +54971,15 @@
       <c r="C108" t="s">
         <v>125</v>
       </c>
+      <c r="E108">
+        <v>4</v>
+      </c>
+      <c r="F108" t="b">
+        <v>0</v>
+      </c>
+      <c r="G108" t="b">
+        <v>0</v>
+      </c>
       <c r="K108" s="1"/>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
@@ -54458,6 +54992,15 @@
       <c r="C109" t="s">
         <v>182</v>
       </c>
+      <c r="E109">
+        <v>4</v>
+      </c>
+      <c r="F109" t="b">
+        <v>0</v>
+      </c>
+      <c r="G109" t="b">
+        <v>0</v>
+      </c>
       <c r="K109" s="1"/>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
@@ -54470,6 +55013,15 @@
       <c r="C110" t="s">
         <v>183</v>
       </c>
+      <c r="E110">
+        <v>5</v>
+      </c>
+      <c r="F110" t="b">
+        <v>0</v>
+      </c>
+      <c r="G110" t="b">
+        <v>1</v>
+      </c>
       <c r="K110" s="1"/>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
@@ -54482,6 +55034,15 @@
       <c r="C111" t="s">
         <v>184</v>
       </c>
+      <c r="E111">
+        <v>4</v>
+      </c>
+      <c r="F111" t="b">
+        <v>0</v>
+      </c>
+      <c r="G111" t="b">
+        <v>0</v>
+      </c>
       <c r="K111" s="1"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
@@ -54494,6 +55055,15 @@
       <c r="C112" t="s">
         <v>123</v>
       </c>
+      <c r="E112">
+        <v>4</v>
+      </c>
+      <c r="F112" t="b">
+        <v>0</v>
+      </c>
+      <c r="G112" t="b">
+        <v>0</v>
+      </c>
       <c r="K112" s="1"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
@@ -54506,6 +55076,15 @@
       <c r="C113" t="s">
         <v>185</v>
       </c>
+      <c r="E113">
+        <v>5</v>
+      </c>
+      <c r="F113" t="b">
+        <v>0</v>
+      </c>
+      <c r="G113" t="b">
+        <v>0</v>
+      </c>
       <c r="K113" s="1"/>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
@@ -54518,6 +55097,15 @@
       <c r="C114" t="s">
         <v>174</v>
       </c>
+      <c r="E114">
+        <v>5</v>
+      </c>
+      <c r="F114" t="b">
+        <v>0</v>
+      </c>
+      <c r="G114" t="b">
+        <v>1</v>
+      </c>
       <c r="K114" s="1"/>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
@@ -54530,6 +55118,15 @@
       <c r="C115" t="s">
         <v>186</v>
       </c>
+      <c r="E115">
+        <v>5</v>
+      </c>
+      <c r="F115" t="b">
+        <v>1</v>
+      </c>
+      <c r="G115" t="b">
+        <v>0</v>
+      </c>
       <c r="K115" s="1"/>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
@@ -54542,6 +55139,15 @@
       <c r="C116" t="s">
         <v>175</v>
       </c>
+      <c r="E116">
+        <v>4</v>
+      </c>
+      <c r="F116" t="b">
+        <v>0</v>
+      </c>
+      <c r="G116" t="b">
+        <v>0</v>
+      </c>
       <c r="K116" s="1"/>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
@@ -54554,6 +55160,15 @@
       <c r="C117" t="s">
         <v>182</v>
       </c>
+      <c r="E117">
+        <v>5</v>
+      </c>
+      <c r="F117" t="b">
+        <v>0</v>
+      </c>
+      <c r="G117" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
@@ -54565,6 +55180,15 @@
       <c r="C118" t="s">
         <v>153</v>
       </c>
+      <c r="E118">
+        <v>5</v>
+      </c>
+      <c r="F118" t="b">
+        <v>0</v>
+      </c>
+      <c r="G118" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
@@ -54576,6 +55200,15 @@
       <c r="C119" t="s">
         <v>195</v>
       </c>
+      <c r="E119">
+        <v>5</v>
+      </c>
+      <c r="F119" t="b">
+        <v>0</v>
+      </c>
+      <c r="G119" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
@@ -54587,6 +55220,15 @@
       <c r="C120" t="s">
         <v>197</v>
       </c>
+      <c r="E120">
+        <v>5</v>
+      </c>
+      <c r="F120" t="b">
+        <v>0</v>
+      </c>
+      <c r="G120" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
@@ -54598,6 +55240,15 @@
       <c r="C121" t="s">
         <v>199</v>
       </c>
+      <c r="E121">
+        <v>5</v>
+      </c>
+      <c r="F121" t="b">
+        <v>0</v>
+      </c>
+      <c r="G121" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
@@ -54609,6 +55260,15 @@
       <c r="C122" t="s">
         <v>199</v>
       </c>
+      <c r="E122">
+        <v>4</v>
+      </c>
+      <c r="F122" t="b">
+        <v>0</v>
+      </c>
+      <c r="G122" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
@@ -54620,6 +55280,15 @@
       <c r="C123" t="s">
         <v>202</v>
       </c>
+      <c r="E123">
+        <v>5</v>
+      </c>
+      <c r="F123" t="b">
+        <v>0</v>
+      </c>
+      <c r="G123" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
@@ -54631,6 +55300,15 @@
       <c r="C124" t="s">
         <v>204</v>
       </c>
+      <c r="E124">
+        <v>5</v>
+      </c>
+      <c r="F124" t="b">
+        <v>0</v>
+      </c>
+      <c r="G124" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
@@ -54642,6 +55320,15 @@
       <c r="C125" t="s">
         <v>206</v>
       </c>
+      <c r="E125">
+        <v>4</v>
+      </c>
+      <c r="F125" t="b">
+        <v>0</v>
+      </c>
+      <c r="G125" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
@@ -54653,6 +55340,15 @@
       <c r="C126" t="s">
         <v>206</v>
       </c>
+      <c r="E126">
+        <v>5</v>
+      </c>
+      <c r="F126" t="b">
+        <v>0</v>
+      </c>
+      <c r="G126" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
@@ -54663,6 +55359,15 @@
       </c>
       <c r="C127" t="s">
         <v>206</v>
+      </c>
+      <c r="E127">
+        <v>4</v>
+      </c>
+      <c r="F127" t="b">
+        <v>0</v>
+      </c>
+      <c r="G127" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>